<commit_message>
feat: initialize 2026 OBE curriculum documentation, reporting tools, and migration audit files
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/024_RINGKAS_EKIVALENSI_UNTUK_AWAM.xlsx
+++ b/KURIKULUM2026_REVISI/024_RINGKAS_EKIVALENSI_UNTUK_AWAM.xlsx
@@ -2019,7 +2019,7 @@
       </c>
       <c r="F26" s="19" t="inlineStr">
         <is>
-          <t>STC-04</t>
+          <t>STC-701</t>
         </is>
       </c>
       <c r="G26" s="20" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>STA-02</t>
+          <t>STA-601</t>
         </is>
       </c>
       <c r="G27" s="20" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="F43" s="19" t="inlineStr">
         <is>
-          <t>STB-01</t>
+          <t>STB-501</t>
         </is>
       </c>
       <c r="G43" s="20" t="inlineStr">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="F45" s="19" t="inlineStr">
         <is>
-          <t>STC-04</t>
+          <t>STC-701</t>
         </is>
       </c>
       <c r="G45" s="20" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="F47" s="19" t="inlineStr">
         <is>
-          <t>STA-01</t>
+          <t>STA-501</t>
         </is>
       </c>
       <c r="G47" s="20" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="F59" s="19" t="inlineStr">
         <is>
-          <t>STB-04</t>
+          <t>STB-701</t>
         </is>
       </c>
       <c r="G59" s="20" t="inlineStr">
@@ -5132,7 +5132,7 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>STA-01</t>
+          <t>STA-501</t>
         </is>
       </c>
       <c r="C39" s="20" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>STB-01</t>
+          <t>STB-501</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>STC-01</t>
+          <t>STC-501</t>
         </is>
       </c>
       <c r="C41" s="20" t="inlineStr">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>STA-02</t>
+          <t>STA-601</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>STA-03</t>
+          <t>STA-602</t>
         </is>
       </c>
       <c r="C49" s="20" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>STB-02</t>
+          <t>STB-601</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>STB-03</t>
+          <t>STB-602</t>
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>STC-02</t>
+          <t>STC-601</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B53" s="19" t="inlineStr">
         <is>
-          <t>STC-03</t>
+          <t>STC-602</t>
         </is>
       </c>
       <c r="C53" s="20" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B61" s="19" t="inlineStr">
         <is>
-          <t>STA-04</t>
+          <t>STA-701</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="B62" s="19" t="inlineStr">
         <is>
-          <t>STA-05</t>
+          <t>STA-702</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="B63" s="19" t="inlineStr">
         <is>
-          <t>STA-06</t>
+          <t>STA-703</t>
         </is>
       </c>
       <c r="C63" s="20" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>STB-04</t>
+          <t>STB-701</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>STB-05</t>
+          <t>STB-702</t>
         </is>
       </c>
       <c r="C65" s="20" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="B66" s="19" t="inlineStr">
         <is>
-          <t>STB-06</t>
+          <t>STB-703</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="B67" s="19" t="inlineStr">
         <is>
-          <t>STC-04</t>
+          <t>STC-701</t>
         </is>
       </c>
       <c r="C67" s="20" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>STC-05</t>
+          <t>STC-702</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="B69" s="19" t="inlineStr">
         <is>
-          <t>STC-06</t>
+          <t>STC-703</t>
         </is>
       </c>
       <c r="C69" s="20" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>STA-01</t>
+          <t>STA-501</t>
         </is>
       </c>
       <c r="D5" s="20" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>STA-02</t>
+          <t>STA-601</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>STA-03</t>
+          <t>STA-602</t>
         </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>STA-04</t>
+          <t>STA-701</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>STA-05</t>
+          <t>STA-702</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>STA-06</t>
+          <t>STA-703</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>STB-01</t>
+          <t>STB-501</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>STB-02</t>
+          <t>STB-601</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -7434,7 +7434,7 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>STB-03</t>
+          <t>STB-602</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>STB-04</t>
+          <t>STB-701</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>STB-05</t>
+          <t>STB-702</t>
         </is>
       </c>
       <c r="D15" s="20" t="inlineStr">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>STB-06</t>
+          <t>STB-703</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>STC-01</t>
+          <t>STC-501</t>
         </is>
       </c>
       <c r="D17" s="20" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>STC-02</t>
+          <t>STC-601</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -7662,7 +7662,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>STC-03</t>
+          <t>STC-602</t>
         </is>
       </c>
       <c r="D19" s="20" t="inlineStr">
@@ -7700,7 +7700,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>STC-04</t>
+          <t>STC-701</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>STC-05</t>
+          <t>STC-702</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -7776,7 +7776,7 @@
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>STC-06</t>
+          <t>STC-703</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>Dua MK mengampu BK yang sama (BK-IS13 / BK-IT09) dengan overlap ± 70%. Materi riset pengguna lanjutan dipindahkan ke elektif `STC-01` UX Research &amp; Design</t>
+          <t>Dua MK mengampu BK yang sama (BK-IS13 / BK-IT09) dengan overlap ± 70%. Materi riset pengguna lanjutan dipindahkan ke elektif `STC-501` UX Research &amp; Design</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>STC-04 Immersive Media &amp; XR Development</t>
+          <t>STC-701 Immersive Media &amp; XR Development</t>
         </is>
       </c>
       <c r="E8" s="18" t="n">

</xml_diff>